<commit_message>
feat: actualiza el modelo de socios
</commit_message>
<xml_diff>
--- a/tests/fixtures/socios-template.xlsx
+++ b/tests/fixtures/socios-template.xlsx
@@ -18,7 +18,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+  <si>
+    <t xml:space="preserve">N° Socio</t>
+  </si>
   <si>
     <t xml:space="preserve">NOMBRE Y APELLIDO</t>
   </si>
@@ -29,13 +32,7 @@
     <t xml:space="preserve">DOCUMENTO DE IDENTIDAD</t>
   </si>
   <si>
-    <t>NACIONALIDAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESTADO CIVIL</t>
-  </si>
-  <si>
-    <t>EDAD</t>
+    <t xml:space="preserve">FECHA de NACIMIENTO</t>
   </si>
   <si>
     <t>TELEFONO</t>
@@ -44,10 +41,16 @@
     <t xml:space="preserve">CARACTER DEL SOCIO</t>
   </si>
   <si>
-    <t xml:space="preserve">FECHA DE INGRESO/ EGRESO</t>
+    <t xml:space="preserve">FECHA DE INGRESO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA DE EGRESO</t>
   </si>
   <si>
     <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
   <si>
     <t>Prueba,Ana</t>
@@ -174,39 +177,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10.000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.000000"/>
-      <color rgb="FFC00000"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="22"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -221,21 +205,15 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" quotePrefix="0" pivotButton="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -761,381 +739,375 @@
   </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="24.7109375"/>
-    <col customWidth="1" min="3" max="3" width="27.28125"/>
-    <col customWidth="1" min="4" max="4" width="28.7109375"/>
-    <col customWidth="1" min="5" max="5" width="20.421875"/>
-    <col customWidth="1" min="6" max="6" width="19.421875"/>
-    <col customWidth="1" min="7" max="7" width="21.140625"/>
-    <col customWidth="1" min="8" max="8" width="13.00390625"/>
-    <col customWidth="1" min="9" max="9" width="13.421875"/>
-    <col customWidth="1" min="10" max="10" width="22.421875"/>
-    <col customWidth="1" min="11" max="11" width="25.8515625"/>
-    <col customWidth="1" min="12" max="12" width="19.57421875"/>
-    <col customWidth="1" min="135" max="135" width="17.8515625"/>
-    <col customWidth="1" hidden="1" min="136" max="136" width="0"/>
-    <col customWidth="1" min="137" max="137" width="26.7109375"/>
+    <col customWidth="1" min="1" max="1" width="24.7109375"/>
+    <col customWidth="1" min="2" max="2" width="27.28125"/>
+    <col customWidth="1" min="3" max="3" width="28.7109375"/>
+    <col customWidth="1" min="4" max="4" width="20.421875"/>
+    <col customWidth="1" min="5" max="5" width="19.421875"/>
+    <col customWidth="1" min="6" max="6" width="21.140625"/>
+    <col customWidth="1" min="7" max="7" width="13.00390625"/>
+    <col customWidth="1" min="8" max="8" width="13.421875"/>
+    <col customWidth="1" min="9" max="9" width="22.421875"/>
+    <col customWidth="1" min="10" max="10" width="25.8515625"/>
+    <col customWidth="1" min="11" max="11" width="19.57421875"/>
+    <col customWidth="1" min="134" max="134" width="17.8515625"/>
+    <col customWidth="1" hidden="1" min="135" max="135" width="0"/>
+    <col customWidth="1" min="136" max="136" width="26.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5">
-      <c r="A1">
+    <row r="1" ht="28.5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="C1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" ht="18.75">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" ht="18.75">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" ht="18.75">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" ht="21">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" ht="21">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" ht="21">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" ht="21">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" ht="21">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" ht="21">
+      <c r="A10">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" ht="18.75">
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" ht="21">
+      <c r="A11">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" ht="18.75">
-      <c r="A3" s="5"/>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" ht="21">
+      <c r="A12">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" ht="18.75">
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" ht="21">
+      <c r="A13">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" ht="21">
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" ht="18.75">
+      <c r="A14">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" ht="21">
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" ht="21">
+      <c r="A15">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" ht="21">
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" ht="21">
+      <c r="A16">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" ht="21">
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" ht="21">
+      <c r="A17">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" ht="21">
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" ht="21">
+      <c r="A18">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" ht="21">
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" ht="21">
+      <c r="A19">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" ht="21">
-      <c r="B11">
-        <v>10</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" ht="21">
+      <c r="A20">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" ht="21">
-      <c r="B12">
-        <v>11</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" ht="21">
+      <c r="A21">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" ht="21">
-      <c r="B13">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" ht="21">
+      <c r="A22">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" ht="18.75">
-      <c r="B14">
-        <v>13</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" ht="21">
+      <c r="A23">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" ht="21">
-      <c r="B15">
-        <v>14</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" ht="21">
+      <c r="A24">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" ht="21">
-      <c r="B16">
-        <v>15</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" ht="18.75">
+      <c r="A25">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" ht="21">
-      <c r="A17" s="5"/>
-      <c r="B17">
-        <v>16</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" ht="21">
+      <c r="A26">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" ht="21">
-      <c r="A18" s="5"/>
-      <c r="B18">
-        <v>17</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" ht="21">
+      <c r="A27">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" ht="21">
-      <c r="B19">
-        <v>18</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" ht="18.75">
+      <c r="A28">
         <v>27</v>
       </c>
-    </row>
-    <row r="20" ht="21">
-      <c r="B20">
-        <v>19</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" ht="18.75">
+      <c r="A29">
         <v>28</v>
       </c>
-    </row>
-    <row r="21" ht="21">
-      <c r="B21">
-        <v>20</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="B29" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" ht="21">
+      <c r="A30">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" ht="21">
-      <c r="B22">
-        <v>21</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" ht="21">
+      <c r="A31">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" ht="21">
-      <c r="B23">
-        <v>22</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="B31" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="32" ht="21">
+      <c r="A32">
         <v>31</v>
       </c>
-    </row>
-    <row r="24" ht="21">
-      <c r="B24">
-        <v>23</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" ht="21">
+      <c r="A33">
         <v>32</v>
       </c>
-    </row>
-    <row r="25" ht="18.75">
-      <c r="B25">
-        <v>24</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="B33" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" ht="21">
+      <c r="A34">
         <v>33</v>
       </c>
-    </row>
-    <row r="26" ht="21">
-      <c r="B26">
-        <v>25</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" ht="21">
+      <c r="A35">
         <v>34</v>
       </c>
-    </row>
-    <row r="27" ht="21">
-      <c r="B27">
-        <v>26</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="B35" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" ht="21">
+      <c r="A36">
         <v>35</v>
       </c>
-    </row>
-    <row r="28" ht="18.75">
-      <c r="B28">
-        <v>27</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="B36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" ht="21">
+      <c r="A37">
         <v>36</v>
       </c>
-    </row>
-    <row r="29" ht="18.75">
-      <c r="A29" s="5"/>
-      <c r="B29">
-        <v>28</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="B37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" ht="21">
+      <c r="A38">
         <v>37</v>
       </c>
-    </row>
-    <row r="30" ht="21">
-      <c r="B30">
-        <v>29</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="B38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" ht="21">
+      <c r="A39">
         <v>38</v>
       </c>
-    </row>
-    <row r="31" ht="21">
-      <c r="B31">
-        <v>30</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40" ht="21">
+      <c r="A40">
         <v>39</v>
       </c>
-    </row>
-    <row r="32" ht="21">
-      <c r="B32">
-        <v>31</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="B40" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" ht="21">
+      <c r="A41">
         <v>40</v>
       </c>
-    </row>
-    <row r="33" ht="21">
-      <c r="B33">
-        <v>32</v>
-      </c>
-      <c r="C33" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="34" ht="21">
-      <c r="B34">
-        <v>33</v>
-      </c>
-      <c r="C34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35" ht="21">
-      <c r="B35">
-        <v>34</v>
-      </c>
-      <c r="C35" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="36" ht="21">
-      <c r="B36">
-        <v>35</v>
-      </c>
-      <c r="C36" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="37" ht="21">
-      <c r="A37" s="5"/>
-      <c r="B37">
-        <v>36</v>
-      </c>
-      <c r="C37" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" ht="21">
-      <c r="B38">
-        <v>37</v>
-      </c>
-      <c r="C38" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="39" ht="21">
-      <c r="B39">
-        <v>38</v>
-      </c>
-      <c r="C39" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="40" ht="21">
-      <c r="B40">
-        <v>39</v>
-      </c>
-      <c r="C40" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="41" ht="21">
-      <c r="B41">
-        <v>40</v>
-      </c>
-      <c r="C41" t="s">
-        <v>49</v>
+      <c r="B41" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="42" ht="21"/>

</xml_diff>

<commit_message>
feat: mejora la insercion de socios y agrega pruebas
</commit_message>
<xml_diff>
--- a/tests/fixtures/socios-template.xlsx
+++ b/tests/fixtures/socios-template.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t xml:space="preserve">N° Socio</t>
   </si>
@@ -164,13 +164,10 @@
     <t>Testigo,Marina</t>
   </si>
   <si>
-    <t>Testigo,Nicolas</t>
+    <t>Testigo,Pedro</t>
   </si>
   <si>
     <t>Testigo,Ofelia</t>
-  </si>
-  <si>
-    <t>Testigo,Pedro</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1085,7 @@
     </row>
     <row r="39" ht="21">
       <c r="A39">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B39" t="s">
         <v>48</v>
@@ -1102,14 +1099,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" ht="21">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>50</v>
-      </c>
-    </row>
+    <row r="41" ht="21"/>
     <row r="42" ht="21"/>
     <row r="43" ht="21"/>
     <row r="44" ht="21"/>

</xml_diff>